<commit_message>
MAJOR: consolidate all models
</commit_message>
<xml_diff>
--- a/foragingModelTable.xlsx
+++ b/foragingModelTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/exs165/Dropbox/foraging/code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEBB6B9A-9E12-CC4B-B6F2-AEABA52BCFB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBC8FCA9-1451-0448-8C14-B578FDCB5930}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11160" yWindow="3980" windowWidth="27240" windowHeight="16440" xr2:uid="{AF09A64C-08B3-A642-B0D0-C38CF1EBFD20}"/>
+    <workbookView xWindow="460" yWindow="500" windowWidth="27240" windowHeight="16320" xr2:uid="{AF09A64C-08B3-A642-B0D0-C38CF1EBFD20}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>